<commit_message>
Ground the proposal in full-source review and validate navigator tasks
</commit_message>
<xml_diff>
--- a/submissions/adriamasnou_methods_description.xlsx
+++ b/submissions/adriamasnou_methods_description.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 1 methods" sheetId="1" r:id="R6b104b45478d42ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 2 methods" sheetId="2" r:id="R409b755051724818"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 1 methods" sheetId="1" r:id="R0634527638ff4685"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 2 methods" sheetId="2" r:id="R938aa0259b5b473f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -616,7 +616,7 @@
     <x:mergeCell ref="A2:B4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1f750105e194455"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra20f7dd029674fec"/>
 </x:worksheet>
 </file>
 
@@ -681,14 +681,14 @@
         <x:v>Both: LLM-assisted literature discovery and structured extraction generated leads; source-by-source review retained, narrowed or rejected claims. Existing mining records include adversarial checks and quote verification, but those checks are not independent clinical validation or an estimate of the final report's error rate. Candidate selection was interpretive, not an automated drug-ranking model. The final proposal distinguishes observed results, cross-model extrapolation and proposed experiments. No clinical expert endorsement is claimed.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="66" hidden="0" customHeight="1">
+    <x:row r="10" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A10" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Please describe any manual literature review or expert curation in detail.</x:t>
         </x:is>
       </x:c>
       <x:c r="B10" s="8" t="str">
-        <x:v>Load-bearing evidence was checked against held primary texts and regulatory documents, including methods, figure legends and the conditions of experiments. New PMID identities were verified with NCBI esummary. The 2026-10-23 revision compared the EMA NPC concentration concerns with Kuta et al.'s lower-concentration murine stress models (PMID 31900865; full main body read, supplements not used for quantitative claims). It removed a blanket ER-compartment exclusion, unsupported clinical contraindication wording, protein/NMD certainties and subjective success probabilities. Paper holdings do not prove every claim has been independently validated; no new aggregate full-text-read count is asserted.</x:v>
+        <x:v>Primary main texts, methods, figures and available supplements were read with explicit coverage records; missing material remains flagged. PMID identities were verified with NCBI esummary. The source pyramid uses Crossref deposited references first, then GROBID residue and co-citation/tier-2 leads. This revision corrected a wrong seed identity, journal-DOI votes and duplicate extraction votes, with regression controls. Kuta dose/time-course supplements, negative ALS/IBM trials, the dependent NPC reanalysis, positive NMN/BubR1 evidence and a 4-PBA/Hsp70 counterexample informed the comparison. Source findings are distinguished from transfer to MVA. No shelf-wide complete-read claim or independent clinical validation is made; see literature-reading-record.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" s="6" customFormat="1" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -708,7 +708,7 @@
         </x:is>
       </x:c>
       <x:c r="B12" s="8" t="str">
-        <x:v>PubMed, Europe PMC and NCBI E-utilities for literature and identifier checks; FDA DailyMed and EMA assessments for regulatory/pharmacology context; ClinVar, gnomAD v4.1, UniProt O60566, OMIM and LOVD for variant/gene evidence; Ensembl VEP, local SpliceAI and Exomiser/HPO for annotation and prioritisation; NIST GIAB HG002 plus a known FGFR2 spike for a computational scale smoke test. The PGT-M navigator uses the HFEA workbook dated 2026-08-05 plus retained ClinVar gene_condition_source_id, HPO genes_to_disease and OMIM mim2gene files. Source SHA-256 hashes, dates and mapping disagreements are supplied. The expert-assertion proxy uses a dated ClinVar variant_summary snapshot. None of these is described as a live registry mirror.</x:v>
+        <x:v>Crossref reference deposits and local GROBID parsing for source-pyramid discovery; PubMed, Europe PMC and NCBI E-utilities for literature and identifier checks; FDA DailyMed and EMA assessments for regulatory/pharmacology context; ClinVar, gnomAD v4.1, UniProt O60566, OMIM and LOVD for variant/gene evidence; Ensembl VEP, local SpliceAI and Exomiser/HPO for annotation and prioritisation; NIST GIAB HG002 plus a known FGFR2 spike for a computational scale smoke test. The PGT-M navigator uses the HFEA workbook dated 2026-08-05 plus retained ClinVar gene_condition_source_id, HPO genes_to_disease and OMIM mim2gene files. Source SHA-256 hashes, dates and mapping disagreements are supplied. The expert-assertion proxy uses a dated ClinVar variant_summary snapshot. None of these is described as a live registry mirror.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -741,7 +741,7 @@
         <x:v>One participant with LLM assistance; project records span 2026-08-26 to 2026-10-23, not continuous full-time effort. Total person-hours and cost were not reliably logged. Historical recorded runs include VEP annotation of 313,417 distinct variants in 10 min 28 s and an Exomiser HG002 spike-in run in 9 min 20 s on a local Apple M3 Max laptop with external databases; these are machine-specific observations, not general runtime guarantees. Prior records identify Anthropic Claude-assisted work; this revision used OpenAI Codex for research, code, drafting and checks. The participant confirms Claude Max 20x and ChatGPT Pro 200 account tiers (23 October 2026). Provider retention settings have not been independently verified. No claim of human clinical expert review is made. No wet-lab experiment, patient treatment or laboratory commitment has occurred.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" s="6" customFormat="1" ht="237.60000610351562" hidden="0" customHeight="1">
+    <x:row r="16" s="6" customFormat="1" ht="250.8000030517578" hidden="0" customHeight="1">
       <x:c r="A16" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Provide a method abstract (up to 500 words). Please include strengths and limitations of your approach as well as methodological detail.</x:t>
@@ -749,8 +749,8 @@
       </x:c>
       <x:c r="B16" s="8" t="str">
         <x:v>We propose arimoclomol as a conditional preclinical repurposing candidate for BUB1B-MVA. The identified p.Leu737* and p.Asn1002Lys variants are consistent with the disease model, but phase is inferred and allele-specific protein consequences are unmeasured. Published BubR1 work motivates testing whether an abundance-limited, functionally rescuable state exists. Regulatory and primary pharmacology evidence makes exposure and cellular context essential limits.
-The proposed experiment compares full-length WT and N1002K at matched abundance, measures protein turnover/localisation and pathway response, and tests chromosome segregation, checkpoint response, proliferation and cell fate. A protein increase, fragment thermal result or high-exposure-only effect cannot establish translational rescue. Failed controls produce an indeterminate result; valid lack of engagement or function rejects the tested drug–exposure–system combination.
-Delivered artifacts include a portable interpretation canary and an offline gene-to-condition navigator with source hashes, per-gene evidence, source disagreements and all unmapped rows. The navigator indexes 2,063 rows of a dated HFEA workbook. Real SpliceAI inference passes six controls; a separate checker self-test rejects nine injected failures. A historical public HG002/FGFR2 spike-in run demonstrates genome-scale execution, not diagnostic sensitivity or freedom from knowledge leakage.
+The proposed experiment compares full-length WT and N1002K at matched abundance, measures protein turnover/localisation and pathway response, and tests chromosome segregation, checkpoint response, proliferation and cell fate. A protein increase, fragment thermal result or high-exposure-only effect cannot establish translational rescue. Failed controls produce an indeterminate result; an upper confidence bound below a prespecified worthwhile functional benefit rejects the tested combination; imprecise results remain inconclusive. A functional hit without HSP engagement requires separate mechanism investigation.
+Delivered artifacts include a portable interpretation canary and an offline gene-to-condition navigator with source hashes, per-gene evidence, source disagreements and all unmapped rows. The navigator indexes 2,063 dated HFEA rows; eleven selected source-adjudicated lookup tasks pass in an unblinded convenience evaluation. Real SpliceAI inference passes six controls; a separate checker self-test rejects nine injected failures. A historical public HG002/FGFR2 spike-in run demonstrates genome-scale execution, not diagnostic sensitivity or freedom from knowledge leakage.
 Strengths are explicit source provenance, separation of inference from measurement and testable advancement criteria. Limitations include no N1002K drug-rescue result, no validated patient-relevant model, no clinical efficacy evidence, no family usability study and incomplete translation from other experimental systems. The work delivers a falsifiable candidate proposal and reusable tools, not a treatment recommendation.</x:v>
       </x:c>
     </x:row>
@@ -759,6 +759,6 @@
     <x:mergeCell ref="A2:B4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R148354366a1b4583"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra88014b13b454df6"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete both methods tabs and clarify retained compute evidence
</commit_message>
<xml_diff>
--- a/submissions/adriamasnou_methods_description.xlsx
+++ b/submissions/adriamasnou_methods_description.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 1 methods" sheetId="1" r:id="R0634527638ff4685"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 2 methods" sheetId="2" r:id="R938aa0259b5b473f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 1 methods" sheetId="1" r:id="Rcfad3070d3f34211"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 2 methods" sheetId="2" r:id="R622ff4def2624213"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -488,8 +488,8 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="85.1640625" style="6" customWidth="1"/>
-    <x:col min="2" max="2" width="45" style="6" customWidth="1"/>
+    <x:col min="1" max="1" width="64" style="6" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="110" style="6" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" s="6" customFormat="1" ht="16" customHeight="1">
@@ -515,108 +515,141 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="2" t="inlineStr">
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Team name</x:t>
         </x:is>
       </x:c>
-      <x:c r="B7" s="3" t="n"/>
-    </x:row>
-    <x:row r="8" s="6" customFormat="1" ht="30" customHeight="1">
-      <x:c r="A8" s="2" t="inlineStr">
+      <x:c r="B7" s="8" t="str">
+        <x:v>adriamasnou</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" s="6" customFormat="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Model number (fill out this form once per model/approach submitted; up to 6)</x:t>
         </x:is>
       </x:c>
-      <x:c r="B8" s="3" t="n"/>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="2" t="inlineStr">
+      <x:c r="B8" s="8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="171.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A9" s="7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Please describe your model/approach in detail.</x:t>
         </x:is>
       </x:c>
-      <x:c r="B9" s="3" t="n"/>
-    </x:row>
-    <x:row r="10" s="6" customFormat="1" ht="45" customHeight="1">
-      <x:c r="A10" s="4" t="inlineStr">
+      <x:c r="B9" s="8" t="str">
+        <x:v>Model 1 was a phenotype-informed, candidate-gene baseline using the organizer-provided GRCh38 GATK VCF and clinical/HPO information. Known MVA genes informed the prior, with BUB1B selected for the targeted computational pass. A Python 3 script streamed the supplied VCF, extracted the BUB1B locus, and screened PASS heterozygous calls whose ID field was empty. The retained report records 14 locus variants, eight heterozygous, with three passing that screen. Empty IDs in this callset's dbSNP138 annotation were a prioritization heuristic, not proof of novelty or population absence.
+The script retrieved public Ensembl exon/CDS information for the canonical BUB1B transcript, mapped positions to coding sequence locally, asserted reference-base agreement, and computed codon consequences. Review of the supplied calls, phenotype fit and ClinVar assertions informed three curated submission rows: the p.Leu737*/p.Asn1002Lys pair, a stop-plus-intronic alternative, and the stop allele alone as a fallback. A proposed pair does not establish trans phase or pathogenicity of the missense/intronic allele.
+This was not an unbiased genome-wide or trained statistical model. FASTQ realignment, independent re-calling, phenotype-blind scanning, VEP, SpliceAI, SV/CNV studies and Exomiser public-case exercises were subsequent work, not components of the original Model 1 submission.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" s="6" customFormat="1" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A10" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Please state whether the submission file is the automated output of your computational approach (preferred), or if it has undergone downstream manual review and curation.</x:t>
         </x:is>
       </x:c>
-      <x:c r="B10" s="3" t="n"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="4" t="inlineStr">
+      <x:c r="B10" s="8" t="str">
+        <x:v>Downstream manual review and curation were used. The targeted script produced locus/consequence summaries, not the final ranked submission CSV. Candidate combinations, order, narrative notes and epcr values were curated. The retained file has three rows with epcr values 0.9, 0.25 and 0.15; these are subjective prioritization scores, not calibrated probabilities or clinical risk estimates. No independent clinical expert validation is claimed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="132" hidden="0" customHeight="1">
+      <x:c r="A11" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Please describe any downstream manual review in detail.</x:t>
         </x:is>
       </x:c>
-      <x:c r="B11" s="3" t="n"/>
-    </x:row>
-    <x:row r="12" s="6" customFormat="1" ht="60" customHeight="1">
-      <x:c r="A12" s="4" t="inlineStr">
+      <x:c r="B11" s="8" t="str">
+        <x:v>Review considered the supplied VCF's filter/genotype and allele-support fields, locally calculated coding consequences, phenotype/gene fit, and public ClinVar evidence. The stop-plus-missense hypothesis was placed first, followed by an alternative second-allele hypothesis involving an intronic call and then a single-stop fallback. The ClinVar assertion for the stop allele and the VUS assertion for a different nucleotide allele encoding the same Asn1002Lys protein change were corroborative context, not a new clinical classification of this exact pair.
+Later review corrected the original CSV's overstatement that missing dbSNP IDs proved absence from dbSNP. The retained gnomAD v4.1 lookup records the exact Asn1002Lys nucleotide allele with AC1; it is not population-absent. Phase remains inferred and unconfirmed. A later alignment audit found an observed maximum properly paired fragment of 1,272 bp and gaps of 6,769 and 4,142 bp between the three ascertained markers. Those reads and that marker set do not establish a connected phase path; this does not rule out additional markers, other evidence or new sequencing. No new phasing analysis was performed for this form. The submitted historical file is preserved, and these corrections do not constitute a resubmission.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" s="6" customFormat="1" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A12" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Please state whether your approach only used publicly available data (preferred) or if proprietary data was also used. If proprietary data were used, where possible, please also include a submission based only on publicly available data.</x:t>
         </x:is>
       </x:c>
-      <x:c r="B12" s="3" t="n"/>
-    </x:row>
-    <x:row r="13" s="6" customFormat="1" ht="30" customHeight="1">
-      <x:c r="A13" s="4" t="inlineStr">
+      <x:c r="B12" s="8" t="str">
+        <x:v>The approach used public reference/annotation resources plus controlled-access challenge data. It therefore was not based exclusively on publicly available data. The restricted inputs were the organizer-provided proband VCF and clinical/HPO information, not a commercial proprietary reference panel. No other proprietary dataset was used. Code and a small number of named candidate findings can be shared; patient-scale inputs cannot be redistributed. Public-case follow-up work is separate from this original submission.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" s="6" customFormat="1" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A13" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Please describe any public data used in detail (e.g., reference panels, population databases, literature).</x:t>
         </x:is>
       </x:c>
-      <x:c r="B13" s="3" t="n"/>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="4" t="inlineStr">
+      <x:c r="B13" s="8" t="str">
+        <x:v>For the original approach: public Ensembl GRCh38 BUB1B gene/transcript information, canonical transcript ENST00000287598 and its CDS/exon structure; HGVS reporting against NM_001211.6; public ClinVar variant/disease assertions; published MVA gene/disease evidence for the phenotype prior; and HPO vocabulary for the clinical terms. The missing-ID screen used the provided VCF's existing dbSNP138 annotation, rather than a fresh population-frequency search. Ensembl requests used public gene/transcript identifiers, with consequence calculation performed locally.
+The original public-resource snapshots and release identifiers were not all fully pinned. gnomAD v4.1, VEP116, SpliceAI, Exomiser and GIAB/phenopacket resources belong to later checks or validation and must not be credited as original Model 1 ranking inputs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A14" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Please describe any proprietary data used in detail.</x:t>
         </x:is>
       </x:c>
-      <x:c r="B14" s="3" t="n"/>
-    </x:row>
-    <x:row r="15" s="6" customFormat="1" ht="30" customHeight="1">
-      <x:c r="A15" s="4" t="inlineStr">
+      <x:c r="B14" s="8" t="str">
+        <x:v>Controlled challenge inputs were the organizer-provided, de-identified single-proband GRCh38 GATK short-variant VCF and associated clinical/HPO information, accessed under challenge terms. No parental genotypes were available to establish phase. The original baseline used the supplied callset as-is and did not realign the challenge FASTQs. No additional proprietary cohort, commercial annotation panel or private training dataset was used. This methods draft contains no raw sequencing data, clinical source document or genotype-scale derivative.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" s="6" customFormat="1" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A15" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Is your approach able to output proposed pairs of compound heterozygous candidate variants, or only single candidate variants?</x:t>
         </x:is>
       </x:c>
-      <x:c r="B15" s="3" t="n"/>
-    </x:row>
-    <x:row r="16" s="6" customFormat="1" ht="30" customHeight="1">
-      <x:c r="A16" s="4" t="inlineStr">
+      <x:c r="B15" s="8" t="str">
+        <x:v>Both proposed compound-heterozygous candidate pairs and single candidates can be represented. The retained submission has two paired rows, with both variant fields populated, and one single-variant fallback with the second set of fields blank. Pair construction and prioritization were curated for this baseline; the targeted script is not a general automated compound-heterozygote ranker. Trans phase is a hypothesis, not an observed result.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" s="6" customFormat="1" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A16" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">How did you handle secondary or incidental findings, if any? (See the finding_type column in your submission.)</x:t>
         </x:is>
       </x:c>
-      <x:c r="B16" s="3" t="n"/>
-    </x:row>
-    <x:row r="17" s="6" customFormat="1" ht="30" customHeight="1">
-      <x:c r="A17" s="4" t="inlineStr">
+      <x:c r="B16" s="8" t="str">
+        <x:v>All three retained submission rows have finding_type=primary. No secondary or incidental finding was submitted. This targeted baseline did not perform a comprehensive secondary-findings screen, so the lack of secondary rows is not evidence that no such findings exist. No additional clinical classification or disclosure is implied. Later secondary-findings governance work is distinct from the original submission procedure.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" s="6" customFormat="1" ht="158.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A17" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Please provide an estimate of run time and cost for your approach (if possible).</x:t>
         </x:is>
       </x:c>
-      <x:c r="B17" s="3" t="n"/>
-    </x:row>
-    <x:row r="18" s="6" customFormat="1" ht="30" customHeight="1">
-      <x:c r="A18" s="4" t="inlineStr">
+      <x:c r="B17" s="8" t="str">
+        <x:v>An end-to-end runtime and total person-hour/cost record for the original baseline was not retained, so a reliable numerical estimate cannot be supplied from these records. The implementation performs one streaming pass through the compressed VCF, retains only the targeted locus calls, and makes a small number of public Ensembl requests. It requires Python 3, with optional truststore, and no model training or large annotation database for this pass. Project hardware is documented as an Apple M3 Max laptop with 14 cores and 36 GB RAM; that is context, not a measured resource profile for Model 1.
+No separately billed cloud compute is recorded for this baseline. Hardware, electricity, review time and LLM-access costs were not apportioned to it. Later logged alignment, VEP and public Exomiser runtimes in methods-and-self-critique.md are separate follow-up costs and are not the runtime of the submitted Model 1.
+Project records include Anthropic Claude-assisted work; this revision used OpenAI Codex. Participant-confirmed account tiers are Claude Max 20x and ChatGPT Pro 200. Provider retention settings were not independently verified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" s="6" customFormat="1" ht="237.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A18" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Provide a method abstract (up to 500 words). Please include strengths and limitations of your method as well as methodological detail.</x:t>
         </x:is>
       </x:c>
-      <x:c r="B18" s="3" t="n"/>
+      <x:c r="B18" s="8" t="str">
+        <x:v>We developed a phenotype-informed BUB1B candidate-prioritization baseline from the organizer-provided GRCh38 GATK VCF and clinical/HPO information. Known MVA genes supplied a strong prior. A Python 3 script streamed the VCF, extracted the BUB1B locus and screened PASS heterozygous variants with empty ID fields in the callset's dbSNP138 annotation. Public Ensembl exon and coding-sequence information supported local consequence calculation, with reference-base checks. Missing identifiers were a screening heuristic rather than evidence of population absence.
+Phenotype fit, VCF evidence, coding consequences and ClinVar context informed a curated three-row submission. The first hypothesis paired p.Leu737* with p.Asn1002Lys. A stop-plus-intronic alternative and a single-stop fallback followed. The approach supports paired and single candidates, but phase remains unconfirmed, and the residual function of Asn1002Lys is unmeasured. Ranking scores were subjective and uncalibrated. All rows were primary findings; no comprehensive secondary-findings screen was performed.
+Strengths include transparent local processing, a small code/dependency footprint, explicit reference checks and a traceable separation between computational extraction and interpretive ranking. Limitations include candidate-gene ascertainment bias, single-case evaluation, reliance on the supplied callset and historical annotations, incomplete original resource pinning, no parental phase confirmation, and no functional or clinical validation of the proposed missense mechanism. The retained leaderboard score is challenge feedback, not independent diagnostic validation.
+Later FASTQ realignment, independent re-calling, phenotype-blind scanning, VEP/SpliceAI annotation and public Exomiser validation were follow-up analyses. They were not used to generate the original Model 1 submission. Current methods text corrects historical novelty and phasing overclaims while preserving the submitted file.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:B4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra20f7dd029674fec"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72210ae7fa3d4802"/>
 </x:worksheet>
 </file>
 
@@ -661,14 +694,14 @@
         <x:v>adriamasnou</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" s="6" customFormat="1" ht="79.19999694824219" hidden="0" customHeight="1">
+    <x:row r="8" s="6" customFormat="1" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A8" s="7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Please describe your approach in detail (how you went from variant/mechanism to candidate medication(s)).</x:t>
         </x:is>
       </x:c>
       <x:c r="B8" s="8" t="str">
-        <x:v>We propose arimoclomol for conditional preclinical testing in BUB1B-MVA. The candidate links reported BubR1 chaperone dependence to a testable stress-response hypothesis, not a demonstrated rescue. We distinguished inferred phase and predicted nonsense-mediated decay from measured protein function. N1002K is uncharacterised experimentally. The plan compares full-length WT and N1002K at matched abundance, qualifies exposure and pathway response, and requires improved chromosome segregation without cytostasis, cell death or selection explaining the result. The labelled NPC exposure is an anchor, not an MVA dose. A fragment thermal assay is supporting evidence only. Sources: PMID 20516114, 22698286, 33207204, 31900865; MIPLYFFA label 2026-03-18 §§1,11–12; main report and functional-rescue-plan.md.</x:v>
+        <x:v>We propose arimoclomol for conditional preclinical testing in BUB1B-MVA. The candidate links reported BubR1 chaperone dependence to a testable stress-response hypothesis, not a demonstrated rescue. We distinguished inferred phase and predicted nonsense-mediated decay from measured protein function. N1002K is uncharacterised experimentally. The plan compares full-length WT and N1002K at matched abundance, qualifies exposure and pathway response, and requires improved chromosome segregation without cytostasis, cell death or selection explaining the result. The labelled NPC exposure is an anchor, not an MVA dose. A fragment thermal assay is supporting evidence only. Sources: PMID 20516114, 22698286, 33207204, 31900865; MIPLYFFA label 2026-03-18 §§1,11–12; main report and functional-rescue-plan.md. A common-endpoint comparison with exposure-qualified 4-PBA and research-only NMN is prespecified for an experimentally rescuable model; treatment-difference confidence intervals, not separate significance tests, would assess comparative benefit. A replicated cellular result requires a justified tissue-output bridge.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -681,14 +714,14 @@
         <x:v>Both: LLM-assisted literature discovery and structured extraction generated leads; source-by-source review retained, narrowed or rejected claims. Existing mining records include adversarial checks and quote verification, but those checks are not independent clinical validation or an estimate of the final report's error rate. Candidate selection was interpretive, not an automated drug-ranking model. The final proposal distinguishes observed results, cross-model extrapolation and proposed experiments. No clinical expert endorsement is claimed.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="79.19999694824219" hidden="0" customHeight="1">
+    <x:row r="10" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A10" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Please describe any manual literature review or expert curation in detail.</x:t>
         </x:is>
       </x:c>
       <x:c r="B10" s="8" t="str">
-        <x:v>Primary main texts, methods, figures and available supplements were read with explicit coverage records; missing material remains flagged. PMID identities were verified with NCBI esummary. The source pyramid uses Crossref deposited references first, then GROBID residue and co-citation/tier-2 leads. This revision corrected a wrong seed identity, journal-DOI votes and duplicate extraction votes, with regression controls. Kuta dose/time-course supplements, negative ALS/IBM trials, the dependent NPC reanalysis, positive NMN/BubR1 evidence and a 4-PBA/Hsp70 counterexample informed the comparison. Source findings are distinguished from transfer to MVA. No shelf-wide complete-read claim or independent clinical validation is made; see literature-reading-record.md.</x:v>
+        <x:v>Primary main texts, methods, figures and available supplements were read with explicit coverage records; missing material remains flagged. PMID identities were verified with NCBI esummary. The source pyramid uses Crossref deposited references first, then GROBID residue and co-citation/tier-2 leads. This revision corrected a wrong seed identity, journal-DOI votes and duplicate extraction votes, with regression controls. Kuta dose/time-course supplements, negative ALS/IBM trials, the dependent NPC reanalysis, positive NMN/BubR1 evidence and a 4-PBA/Hsp70 counterexample informed the comparison. Three additional direct primary experiments show context-dependent arimoclomol responses and negative protein-trafficking results (PMIDs 38570009, 42283221, 34481829). Original public-case papers were adjudicated separately from phenopacket labels, with conflicts and missing components retained. Source findings are distinguished from transfer to MVA. No shelf-wide complete-read claim or independent clinical validation is made; see literature-reading-record.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" s="6" customFormat="1" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -701,14 +734,14 @@
         <x:v>Public drug/target resources and published literature were used for repurposing evidence; no proprietary drug-target database was used. Some published full texts were accessed through institutional subscriptions. Separately, the challenge's gated patient sequencing and clinical material informed the variant analysis under challenge terms. Those restricted inputs are not redistributed. Public-data derivatives used by the navigator and canary are clearly separated from patient-scale inputs.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" s="6" customFormat="1" ht="79.19999694824219" hidden="0" customHeight="1">
+    <x:row r="12" s="6" customFormat="1" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A12" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Please describe the public data sources used in detail (e.g., DrugBank, ChEMBL, ClinicalTrials.gov, OMIM, PubMed literature search).</x:t>
         </x:is>
       </x:c>
       <x:c r="B12" s="8" t="str">
-        <x:v>Crossref reference deposits and local GROBID parsing for source-pyramid discovery; PubMed, Europe PMC and NCBI E-utilities for literature and identifier checks; FDA DailyMed and EMA assessments for regulatory/pharmacology context; ClinVar, gnomAD v4.1, UniProt O60566, OMIM and LOVD for variant/gene evidence; Ensembl VEP, local SpliceAI and Exomiser/HPO for annotation and prioritisation; NIST GIAB HG002 plus a known FGFR2 spike for a computational scale smoke test. The PGT-M navigator uses the HFEA workbook dated 2026-08-05 plus retained ClinVar gene_condition_source_id, HPO genes_to_disease and OMIM mim2gene files. Source SHA-256 hashes, dates and mapping disagreements are supplied. The expert-assertion proxy uses a dated ClinVar variant_summary snapshot. None of these is described as a live registry mirror.</x:v>
+        <x:v>Crossref reference deposits and local GROBID parsing for source-pyramid discovery; PubMed, Europe PMC and NCBI E-utilities for literature and identifier checks; FDA DailyMed and EMA assessments for regulatory/pharmacology context; ClinVar, gnomAD v4.1, UniProt O60566, OMIM and LOVD for variant/gene evidence; Ensembl VEP, local SpliceAI and Exomiser/HPO for annotation and prioritisation; NIST GIAB HG002/HG001 v4.2.1 GRCh38, Ensembl 116 exons and Phenopacket Store 0.1.19 for a frozen twelve-case, four-arm semi-synthetic evaluation, plus a separately reconstructed FGFR2 scale example. The multi-case evaluation is running; only completed results with execution records will be reported. Preparation alone does not establish recovery. The PGT-M navigator uses the HFEA workbook dated 2026-08-05 plus retained ClinVar gene_condition_source_id, HPO genes_to_disease and OMIM mim2gene files. Source SHA-256 hashes, dates and mapping disagreements are supplied. The expert-assertion proxy uses a dated ClinVar variant_summary snapshot. None of these is described as a live registry mirror.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -731,17 +764,17 @@
         <x:v>The findings are BUB1B c.2210T&gt;G (p.Leu737*) and c.3006T&gt;G (p.Asn1002Lys). Phase is inferred. NMD of this exact stop allele and N1002K abundance/function are unmeasured. The proposed mechanism concerns BubR1 stability and non-catalytic chromosome-segregation/checkpoint functions (PMID 20516114, 22698286, 33207204). Abundance-limited, function-limited, mixed and indeterminate states are experimental categories, not assigned diagnoses. In-silico predictions and a low local splice score do not substitute for functional evidence. A previous bulk-WGS mosaicism claim was withdrawn after read-mapping correction. No clinical reclassification or treatment follows from this work alone.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" s="6" customFormat="1" ht="79.19999694824219" hidden="0" customHeight="1">
+    <x:row r="15" s="6" customFormat="1" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A15" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Please provide an estimate of time or effort spent on this analysis (if possible).</x:t>
         </x:is>
       </x:c>
       <x:c r="B15" s="8" t="str">
-        <x:v>One participant with LLM assistance; project records span 2026-08-26 to 2026-10-23, not continuous full-time effort. Total person-hours and cost were not reliably logged. Historical recorded runs include VEP annotation of 313,417 distinct variants in 10 min 28 s and an Exomiser HG002 spike-in run in 9 min 20 s on a local Apple M3 Max laptop with external databases; these are machine-specific observations, not general runtime guarantees. Prior records identify Anthropic Claude-assisted work; this revision used OpenAI Codex for research, code, drafting and checks. The participant confirms Claude Max 20x and ChatGPT Pro 200 account tiers (23 October 2026). Provider retention settings have not been independently verified. No claim of human clinical expert review is made. No wet-lab experiment, patient treatment or laboratory commitment has occurred.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" s="6" customFormat="1" ht="250.8000030517578" hidden="0" customHeight="1">
+        <x:v>One participant with LLM assistance; project records span 2026-08-26 to 2026-10-24, not continuous full-time effort. Total person-hours and cost were not reliably logged. Historical recorded runs include VEP annotation of 313,417 distinct variants in 10 min 28 s and an Exomiser HG002 spike-in run in 9 min 20 s on a local Apple M3 Max laptop with external databases; The new two-job FGFR2 reconstruction completed in 200.48 s including startup, with FGFR2 first among 2 and 471 scored genes. The August configuration was not recovered. These are machine-specific observations with different settings, not general runtime or accuracy improvements. Prior records identify Anthropic Claude-assisted work; this revision used OpenAI Codex for research, code, drafting and checks. The participant confirms Claude Max 20x and ChatGPT Pro 200 account tiers (23 October 2026). Provider retention settings have not been independently verified. No claim of human clinical expert review is made. No wet-lab experiment, patient treatment or laboratory commitment has occurred.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" s="6" customFormat="1" ht="277.20001220703125" hidden="0" customHeight="1">
       <x:c r="A16" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Provide a method abstract (up to 500 words). Please include strengths and limitations of your approach as well as methodological detail.</x:t>
@@ -750,7 +783,7 @@
       <x:c r="B16" s="8" t="str">
         <x:v>We propose arimoclomol as a conditional preclinical repurposing candidate for BUB1B-MVA. The identified p.Leu737* and p.Asn1002Lys variants are consistent with the disease model, but phase is inferred and allele-specific protein consequences are unmeasured. Published BubR1 work motivates testing whether an abundance-limited, functionally rescuable state exists. Regulatory and primary pharmacology evidence makes exposure and cellular context essential limits.
 The proposed experiment compares full-length WT and N1002K at matched abundance, measures protein turnover/localisation and pathway response, and tests chromosome segregation, checkpoint response, proliferation and cell fate. A protein increase, fragment thermal result or high-exposure-only effect cannot establish translational rescue. Failed controls produce an indeterminate result; an upper confidence bound below a prespecified worthwhile functional benefit rejects the tested combination; imprecise results remain inconclusive. A functional hit without HSP engagement requires separate mechanism investigation.
-Delivered artifacts include a portable interpretation canary and an offline gene-to-condition navigator with source hashes, per-gene evidence, source disagreements and all unmapped rows. The navigator indexes 2,063 dated HFEA rows; eleven selected source-adjudicated lookup tasks pass in an unblinded convenience evaluation. Real SpliceAI inference passes six controls; a separate checker self-test rejects nine injected failures. A historical public HG002/FGFR2 spike-in run demonstrates genome-scale execution, not diagnostic sensitivity or freedom from knowledge leakage.
+Delivered artifacts include a portable interpretation canary and an offline gene-to-condition navigator with source hashes, per-gene evidence, source disagreements and all unmapped rows. The navigator indexes 2,063 dated HFEA rows; 28 frozen queries pass after complete review of all 47 returned row–gene associations. The audit found and repaired 11 lost source qualifiers; this shared-source developer evaluation does not establish clinical validity. Real SpliceAI inference passes six controls; a separate checker self-test rejects nine injected failures. The rescue-decision prototype passes 40 frozen synthetic cases and detects 7 deliberately introduced rule faults. These measure software decisions, not biology. A separately retained public-data evaluation distinguishes source-gene ranking from contributing alleles, phenotype knowledge and diagnostic accuracy.
 Strengths are explicit source provenance, separation of inference from measurement and testable advancement criteria. Limitations include no N1002K drug-rescue result, no validated patient-relevant model, no clinical efficacy evidence, no family usability study and incomplete translation from other experimental systems. The work delivers a falsifiable candidate proposal and reusable tools, not a treatment recommendation.</x:v>
       </x:c>
     </x:row>
@@ -759,6 +792,6 @@
     <x:mergeCell ref="A2:B4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra88014b13b454df6"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77895feb3de3479f"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Deliver paired public validation and phenotype comparator with portable evidence
</commit_message>
<xml_diff>
--- a/submissions/adriamasnou_methods_description.xlsx
+++ b/submissions/adriamasnou_methods_description.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 1 methods" sheetId="1" r:id="Rcfad3070d3f34211"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 2 methods" sheetId="2" r:id="R622ff4def2624213"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 1 methods" sheetId="1" r:id="R979f2017fcf24ac3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 2 methods" sheetId="2" r:id="R26daf1d5cc4944cf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -649,7 +649,7 @@
     <x:mergeCell ref="A2:B4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72210ae7fa3d4802"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08dfd7957f2b4f7a"/>
 </x:worksheet>
 </file>
 
@@ -734,14 +734,14 @@
         <x:v>Public drug/target resources and published literature were used for repurposing evidence; no proprietary drug-target database was used. Some published full texts were accessed through institutional subscriptions. Separately, the challenge's gated patient sequencing and clinical material informed the variant analysis under challenge terms. Those restricted inputs are not redistributed. Public-data derivatives used by the navigator and canary are clearly separated from patient-scale inputs.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" s="6" customFormat="1" ht="105.5999984741211" hidden="0" customHeight="1">
+    <x:row r="12" s="6" customFormat="1" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A12" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Please describe the public data sources used in detail (e.g., DrugBank, ChEMBL, ClinicalTrials.gov, OMIM, PubMed literature search).</x:t>
         </x:is>
       </x:c>
       <x:c r="B12" s="8" t="str">
-        <x:v>Crossref reference deposits and local GROBID parsing for source-pyramid discovery; PubMed, Europe PMC and NCBI E-utilities for literature and identifier checks; FDA DailyMed and EMA assessments for regulatory/pharmacology context; ClinVar, gnomAD v4.1, UniProt O60566, OMIM and LOVD for variant/gene evidence; Ensembl VEP, local SpliceAI and Exomiser/HPO for annotation and prioritisation; NIST GIAB HG002/HG001 v4.2.1 GRCh38, Ensembl 116 exons and Phenopacket Store 0.1.19 for a frozen twelve-case, four-arm semi-synthetic evaluation, plus a separately reconstructed FGFR2 scale example. The multi-case evaluation is running; only completed results with execution records will be reported. Preparation alone does not establish recovery. The PGT-M navigator uses the HFEA workbook dated 2026-08-05 plus retained ClinVar gene_condition_source_id, HPO genes_to_disease and OMIM mim2gene files. Source SHA-256 hashes, dates and mapping disagreements are supplied. The expert-assertion proxy uses a dated ClinVar variant_summary snapshot. None of these is described as a live registry mirror.</x:v>
+        <x:v>Crossref reference deposits and local GROBID parsing for source-pyramid discovery; PubMed, Europe PMC and NCBI E-utilities for literature and identifier checks; FDA DailyMed and EMA assessments for regulatory/pharmacology context; ClinVar, gnomAD v4.1, UniProt O60566, OMIM and LOVD for variant/gene evidence; Ensembl VEP, local SpliceAI and Exomiser/HPO for annotation and prioritisation; NIST GIAB HG002/HG001 v4.2.1 GRCh38, Ensembl 116 exons and Phenopacket Store 0.1.19 for a frozen twelve-case, four-arm semi-synthetic evaluation, plus a separately reconstructed FGFR2 scale example. Both 48-job genome-background batches completed. With original HPO, source-gene top-1/5/10 counts were 6/7/8 of nine primary labels on HG002 and 7/8/8 on HG001. They are the same nine labels, not eighteen independent cases. Five labels retain source qualifications; PAX4 and two X cases remain separate. All four phenotype arms and exact-allele evidence are retained in public-validation.md. The separate original-HPO-only comparator ranked 4/8/8 of nine source genes within 1/5/10 among 19,192 genes; its different candidate universe prevents a causal estimate of sequencing value. This is constructed source-label recovery, not clinical accuracy. The PGT-M navigator uses the HFEA workbook dated 2026-08-05 plus retained ClinVar gene_condition_source_id, HPO genes_to_disease and OMIM mim2gene files. Source SHA-256 hashes, dates and mapping disagreements are supplied. The expert-assertion proxy uses a dated ClinVar variant_summary snapshot. None of these is described as a live registry mirror.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -764,17 +764,17 @@
         <x:v>The findings are BUB1B c.2210T&gt;G (p.Leu737*) and c.3006T&gt;G (p.Asn1002Lys). Phase is inferred. NMD of this exact stop allele and N1002K abundance/function are unmeasured. The proposed mechanism concerns BubR1 stability and non-catalytic chromosome-segregation/checkpoint functions (PMID 20516114, 22698286, 33207204). Abundance-limited, function-limited, mixed and indeterminate states are experimental categories, not assigned diagnoses. In-silico predictions and a low local splice score do not substitute for functional evidence. A previous bulk-WGS mosaicism claim was withdrawn after read-mapping correction. No clinical reclassification or treatment follows from this work alone.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" s="6" customFormat="1" ht="105.5999984741211" hidden="0" customHeight="1">
+    <x:row r="15" s="6" customFormat="1" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A15" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Please provide an estimate of time or effort spent on this analysis (if possible).</x:t>
         </x:is>
       </x:c>
       <x:c r="B15" s="8" t="str">
-        <x:v>One participant with LLM assistance; project records span 2026-08-26 to 2026-10-24, not continuous full-time effort. Total person-hours and cost were not reliably logged. Historical recorded runs include VEP annotation of 313,417 distinct variants in 10 min 28 s and an Exomiser HG002 spike-in run in 9 min 20 s on a local Apple M3 Max laptop with external databases; The new two-job FGFR2 reconstruction completed in 200.48 s including startup, with FGFR2 first among 2 and 471 scored genes. The August configuration was not recovered. These are machine-specific observations with different settings, not general runtime or accuracy improvements. Prior records identify Anthropic Claude-assisted work; this revision used OpenAI Codex for research, code, drafting and checks. The participant confirms Claude Max 20x and ChatGPT Pro 200 account tiers (23 October 2026). Provider retention settings have not been independently verified. No claim of human clinical expert review is made. No wet-lab experiment, patient treatment or laboratory commitment has occurred.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" s="6" customFormat="1" ht="277.20001220703125" hidden="0" customHeight="1">
+        <x:v>One participant with LLM assistance; project records span 2026-08-26 to 2026-10-24, not continuous full-time effort. Total person-hours and cost were not reliably logged. Historical recorded runs include VEP annotation of 313,417 distinct variants in 10 min 28 s and an Exomiser HG002 spike-in run in 9 min 20 s on a local Apple M3 Max laptop with external databases; the new two-job FGFR2 reconstruction completed in 200.48 s including startup, with FGFR2 first among 2 and 471 scored genes. The August configuration was not recovered. The 48-job HG002 and HG001 batches took 3,488.41 and 3,607.42 seconds respectively, including each JVM startup and excluding input preparation/downloads. Their conservative ranks are retained with exact runtime configurations. These are machine-specific observations with different settings, not general runtime or accuracy improvements. Prior records identify Anthropic Claude-assisted work; this revision used OpenAI Codex for research, code, drafting and checks. The participant confirms Claude Max 20x and ChatGPT Pro 200 account tiers (23 October 2026). Provider retention settings have not been independently verified. No claim of human clinical expert review is made. No wet-lab experiment, patient treatment or laboratory commitment has occurred.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" s="6" customFormat="1" ht="290.3999938964844" hidden="0" customHeight="1">
       <x:c r="A16" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Provide a method abstract (up to 500 words). Please include strengths and limitations of your approach as well as methodological detail.</x:t>
@@ -783,7 +783,7 @@
       <x:c r="B16" s="8" t="str">
         <x:v>We propose arimoclomol as a conditional preclinical repurposing candidate for BUB1B-MVA. The identified p.Leu737* and p.Asn1002Lys variants are consistent with the disease model, but phase is inferred and allele-specific protein consequences are unmeasured. Published BubR1 work motivates testing whether an abundance-limited, functionally rescuable state exists. Regulatory and primary pharmacology evidence makes exposure and cellular context essential limits.
 The proposed experiment compares full-length WT and N1002K at matched abundance, measures protein turnover/localisation and pathway response, and tests chromosome segregation, checkpoint response, proliferation and cell fate. A protein increase, fragment thermal result or high-exposure-only effect cannot establish translational rescue. Failed controls produce an indeterminate result; an upper confidence bound below a prespecified worthwhile functional benefit rejects the tested combination; imprecise results remain inconclusive. A functional hit without HSP engagement requires separate mechanism investigation.
-Delivered artifacts include a portable interpretation canary and an offline gene-to-condition navigator with source hashes, per-gene evidence, source disagreements and all unmapped rows. The navigator indexes 2,063 dated HFEA rows; 28 frozen queries pass after complete review of all 47 returned row–gene associations. The audit found and repaired 11 lost source qualifiers; this shared-source developer evaluation does not establish clinical validity. Real SpliceAI inference passes six controls; a separate checker self-test rejects nine injected failures. The rescue-decision prototype passes 40 frozen synthetic cases and detects 7 deliberately introduced rule faults. These measure software decisions, not biology. A separately retained public-data evaluation distinguishes source-gene ranking from contributing alleles, phenotype knowledge and diagnostic accuracy.
+Delivered artifacts include a portable interpretation canary and an offline gene-to-condition navigator with source hashes, per-gene evidence, source disagreements and all unmapped rows. The navigator indexes 2,063 dated HFEA rows; 28 frozen queries pass after complete review of all 47 returned row–gene associations. The audit found and repaired 11 lost source qualifiers; this shared-source developer evaluation does not establish clinical validity. Real SpliceAI inference passes six controls; a separate checker self-test rejects nine injected failures. The rescue-decision prototype passes 40 frozen synthetic cases and detects 7 deliberately introduced rule faults. These measure software decisions, not biology. A 96-job public-data evaluation recovered eight of nine primary source genes within the top ten under original HPO on each of two genome backgrounds. These constructed cases retain source qualifications; gene rank is distinct from joint-allele support, phase and diagnostic accuracy.
 Strengths are explicit source provenance, separation of inference from measurement and testable advancement criteria. Limitations include no N1002K drug-rescue result, no validated patient-relevant model, no clinical efficacy evidence, no family usability study and incomplete translation from other experimental systems. The work delivers a falsifiable candidate proposal and reusable tools, not a treatment recommendation.</x:v>
       </x:c>
     </x:row>
@@ -792,6 +792,6 @@
     <x:mergeCell ref="A2:B4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77895feb3de3479f"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc8c09ae8fac4e3f"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Qualify phenotype gene identities and preserve independent audits
</commit_message>
<xml_diff>
--- a/submissions/adriamasnou_methods_description.xlsx
+++ b/submissions/adriamasnou_methods_description.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 1 methods" sheetId="1" r:id="R979f2017fcf24ac3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 2 methods" sheetId="2" r:id="R26daf1d5cc4944cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 1 methods" sheetId="1" r:id="Refa02fcd6a6c411f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 2 methods" sheetId="2" r:id="R6d48e4d1b1e24472"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -649,7 +649,7 @@
     <x:mergeCell ref="A2:B4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08dfd7957f2b4f7a"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15f8b9730a5e44ea"/>
 </x:worksheet>
 </file>
 
@@ -741,7 +741,7 @@
         </x:is>
       </x:c>
       <x:c r="B12" s="8" t="str">
-        <x:v>Crossref reference deposits and local GROBID parsing for source-pyramid discovery; PubMed, Europe PMC and NCBI E-utilities for literature and identifier checks; FDA DailyMed and EMA assessments for regulatory/pharmacology context; ClinVar, gnomAD v4.1, UniProt O60566, OMIM and LOVD for variant/gene evidence; Ensembl VEP, local SpliceAI and Exomiser/HPO for annotation and prioritisation; NIST GIAB HG002/HG001 v4.2.1 GRCh38, Ensembl 116 exons and Phenopacket Store 0.1.19 for a frozen twelve-case, four-arm semi-synthetic evaluation, plus a separately reconstructed FGFR2 scale example. Both 48-job genome-background batches completed. With original HPO, source-gene top-1/5/10 counts were 6/7/8 of nine primary labels on HG002 and 7/8/8 on HG001. They are the same nine labels, not eighteen independent cases. Five labels retain source qualifications; PAX4 and two X cases remain separate. All four phenotype arms and exact-allele evidence are retained in public-validation.md. The separate original-HPO-only comparator ranked 4/8/8 of nine source genes within 1/5/10 among 19,192 genes; its different candidate universe prevents a causal estimate of sequencing value. This is constructed source-label recovery, not clinical accuracy. The PGT-M navigator uses the HFEA workbook dated 2026-08-05 plus retained ClinVar gene_condition_source_id, HPO genes_to_disease and OMIM mim2gene files. Source SHA-256 hashes, dates and mapping disagreements are supplied. The expert-assertion proxy uses a dated ClinVar variant_summary snapshot. None of these is described as a live registry mirror.</x:v>
+        <x:v>Crossref reference deposits and local GROBID parsing for source-pyramid discovery; PubMed, Europe PMC and NCBI E-utilities for literature and identifier checks; FDA DailyMed and EMA assessments for regulatory/pharmacology context; ClinVar, gnomAD v4.1, UniProt O60566, OMIM and LOVD for variant/gene evidence; Ensembl VEP, local SpliceAI and Exomiser/HPO for annotation and prioritisation; NIST GIAB HG002/HG001 v4.2.1 GRCh38, Ensembl 116 exons and Phenopacket Store 0.1.19 for a frozen twelve-case, four-arm semi-synthetic evaluation, plus a separately reconstructed FGFR2 scale example. Both 48-job genome-background batches completed. With original HPO, source-gene top-1/5/10 counts were 6/7/8 of nine primary labels on HG002 and 7/8/8 on HG001. They are the same nine labels, not eighteen independent cases. Five labels retain source qualifications; PAX4 and two X cases remain separate. All four phenotype arms and exact-allele evidence are retained in public-validation.md. The separate original-HPO-only comparator ranked 4/8/8 of nine source genes within 1/5/10 among 19,192 gene-symbol records (19,116 Entrez IDs; collapsing shared IDs leaves target ranks unchanged); its different candidate universe prevents a causal estimate of sequencing value. This is constructed source-label recovery, not clinical accuracy. The PGT-M navigator uses the HFEA workbook dated 2026-08-05 plus retained ClinVar gene_condition_source_id, HPO genes_to_disease and OMIM mim2gene files. Source SHA-256 hashes, dates and mapping disagreements are supplied. The expert-assertion proxy uses a dated ClinVar variant_summary snapshot. None of these is described as a live registry mirror.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -792,6 +792,6 @@
     <x:mergeCell ref="A2:B4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc8c09ae8fac4e3f"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb47e2a24c2ad4be1"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Deliver independently verified compact benchmark and completed review documents
</commit_message>
<xml_diff>
--- a/submissions/adriamasnou_methods_description.xlsx
+++ b/submissions/adriamasnou_methods_description.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 1 methods" sheetId="1" r:id="Refa02fcd6a6c411f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 2 methods" sheetId="2" r:id="R6d48e4d1b1e24472"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 1 methods" sheetId="1" r:id="R25cdb1bd081b4fde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 2 methods" sheetId="2" r:id="R4dd9b131704741ee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -649,7 +649,7 @@
     <x:mergeCell ref="A2:B4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15f8b9730a5e44ea"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48556272d9de48fa"/>
 </x:worksheet>
 </file>
 
@@ -734,14 +734,14 @@
         <x:v>Public drug/target resources and published literature were used for repurposing evidence; no proprietary drug-target database was used. Some published full texts were accessed through institutional subscriptions. Separately, the challenge's gated patient sequencing and clinical material informed the variant analysis under challenge terms. Those restricted inputs are not redistributed. Public-data derivatives used by the navigator and canary are clearly separated from patient-scale inputs.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" s="6" customFormat="1" ht="158.39999389648438" hidden="0" customHeight="1">
+    <x:row r="12" s="6" customFormat="1" ht="211.1999969482422" hidden="0" customHeight="1">
       <x:c r="A12" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Please describe the public data sources used in detail (e.g., DrugBank, ChEMBL, ClinicalTrials.gov, OMIM, PubMed literature search).</x:t>
         </x:is>
       </x:c>
       <x:c r="B12" s="8" t="str">
-        <x:v>Crossref reference deposits and local GROBID parsing for source-pyramid discovery; PubMed, Europe PMC and NCBI E-utilities for literature and identifier checks; FDA DailyMed and EMA assessments for regulatory/pharmacology context; ClinVar, gnomAD v4.1, UniProt O60566, OMIM and LOVD for variant/gene evidence; Ensembl VEP, local SpliceAI and Exomiser/HPO for annotation and prioritisation; NIST GIAB HG002/HG001 v4.2.1 GRCh38, Ensembl 116 exons and Phenopacket Store 0.1.19 for a frozen twelve-case, four-arm semi-synthetic evaluation, plus a separately reconstructed FGFR2 scale example. Both 48-job genome-background batches completed. With original HPO, source-gene top-1/5/10 counts were 6/7/8 of nine primary labels on HG002 and 7/8/8 on HG001. They are the same nine labels, not eighteen independent cases. Five labels retain source qualifications; PAX4 and two X cases remain separate. All four phenotype arms and exact-allele evidence are retained in public-validation.md. The separate original-HPO-only comparator ranked 4/8/8 of nine source genes within 1/5/10 among 19,192 gene-symbol records (19,116 Entrez IDs; collapsing shared IDs leaves target ranks unchanged); its different candidate universe prevents a causal estimate of sequencing value. This is constructed source-label recovery, not clinical accuracy. The PGT-M navigator uses the HFEA workbook dated 2026-08-05 plus retained ClinVar gene_condition_source_id, HPO genes_to_disease and OMIM mim2gene files. Source SHA-256 hashes, dates and mapping disagreements are supplied. The expert-assertion proxy uses a dated ClinVar variant_summary snapshot. None of these is described as a live registry mirror.</x:v>
+        <x:v>Crossref reference deposits and local GROBID parsing for source-pyramid discovery; PubMed, Europe PMC and NCBI E-utilities for literature and identifier checks; FDA DailyMed and EMA assessments for regulatory/pharmacology context; ClinVar, gnomAD v4.1, UniProt O60566, OMIM and LOVD for variant/gene evidence; Ensembl VEP, local SpliceAI and Exomiser/HPO for annotation and prioritisation; NIST GIAB HG002/HG001 v4.2.1 GRCh38, Ensembl 116 exons and Phenopacket Store 0.1.19 for a frozen twelve-case, four-arm semi-synthetic evaluation, plus a separately reconstructed FGFR2 scale example. Both 48-job genome-background batches completed. With original HPO, source-gene top-1/5/10 counts were 6/7/8 of nine primary labels on HG002 and 7/8/8 on HG001. They are the same nine labels, not eighteen independent cases. Five labels retain source qualifications; PAX4 and two X cases remain separate. All four phenotype arms and exact-allele evidence are retained in public-validation.md. The separate original-HPO-only comparator ranked 4/8/8 of nine source genes within 1/5/10 among 19,192 gene-symbol records (19,116 Entrez IDs; collapsing shared IDs leaves target ranks unchanged); its different candidate universe prevents a causal estimate of sequencing value. This is constructed source-label recovery, not clinical accuracy. A separate compact source-label extension completed 1,418 jobs across 713 signatures, with a fixed autosomal primary denominator of 681. Original-HPO top-1 was 556/681 versus 430/681 without HPO after a disclosed serialization-parser correction; both evaluations are retained. Ten constructed hypotheses per case, current database knowledge and 321 unread source papers prevent clinical-accuracy or competitor-superiority claims. See compact-public-validation.md. The PGT-M navigator uses the HFEA workbook dated 2026-08-05 plus retained ClinVar gene_condition_source_id, HPO genes_to_disease and OMIM mim2gene files. Source SHA-256 hashes, dates and mapping disagreements are supplied. The expert-assertion proxy uses a dated ClinVar variant_summary snapshot. None of these is described as a live registry mirror.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -764,14 +764,14 @@
         <x:v>The findings are BUB1B c.2210T&gt;G (p.Leu737*) and c.3006T&gt;G (p.Asn1002Lys). Phase is inferred. NMD of this exact stop allele and N1002K abundance/function are unmeasured. The proposed mechanism concerns BubR1 stability and non-catalytic chromosome-segregation/checkpoint functions (PMID 20516114, 22698286, 33207204). Abundance-limited, function-limited, mixed and indeterminate states are experimental categories, not assigned diagnoses. In-silico predictions and a low local splice score do not substitute for functional evidence. A previous bulk-WGS mosaicism claim was withdrawn after read-mapping correction. No clinical reclassification or treatment follows from this work alone.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" s="6" customFormat="1" ht="118.80000305175781" hidden="0" customHeight="1">
+    <x:row r="15" s="6" customFormat="1" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A15" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Please provide an estimate of time or effort spent on this analysis (if possible).</x:t>
         </x:is>
       </x:c>
       <x:c r="B15" s="8" t="str">
-        <x:v>One participant with LLM assistance; project records span 2026-08-26 to 2026-10-24, not continuous full-time effort. Total person-hours and cost were not reliably logged. Historical recorded runs include VEP annotation of 313,417 distinct variants in 10 min 28 s and an Exomiser HG002 spike-in run in 9 min 20 s on a local Apple M3 Max laptop with external databases; the new two-job FGFR2 reconstruction completed in 200.48 s including startup, with FGFR2 first among 2 and 471 scored genes. The August configuration was not recovered. The 48-job HG002 and HG001 batches took 3,488.41 and 3,607.42 seconds respectively, including each JVM startup and excluding input preparation/downloads. Their conservative ranks are retained with exact runtime configurations. These are machine-specific observations with different settings, not general runtime or accuracy improvements. Prior records identify Anthropic Claude-assisted work; this revision used OpenAI Codex for research, code, drafting and checks. The participant confirms Claude Max 20x and ChatGPT Pro 200 account tiers (23 October 2026). Provider retention settings have not been independently verified. No claim of human clinical expert review is made. No wet-lab experiment, patient treatment or laboratory commitment has occurred.</x:v>
+        <x:v>One participant with LLM assistance; project records span 2026-08-26 to 2026-10-24, not continuous full-time effort. Total person-hours and cost were not reliably logged. Historical recorded runs include VEP annotation of 313,417 distinct variants in 10 min 28 s and an Exomiser HG002 spike-in run in 9 min 20 s on a local Apple M3 Max laptop with external databases; the new two-job FGFR2 reconstruction completed in 200.48 s including startup, with FGFR2 first among 2 and 471 scored genes. The August configuration was not recovered. The 48-job HG002 and HG001 batches took 3,488.41 and 3,607.42 seconds respectively, including each JVM startup and excluding input preparation/downloads. Their conservative ranks are retained with exact runtime configurations. These are machine-specific observations with different settings, not general runtime or accuracy improvements. Prior records identify Anthropic Claude-assisted work; this revision used OpenAI Codex for research, code, drafting and checks. The participant confirms Claude Max 20x and ChatGPT Pro 200 account tiers (23 October 2026). Provider retention settings have not been independently verified. No claim of human clinical expert review is made. No wet-lab experiment, patient treatment or laboratory commitment has occurred. The separate compact extension completed 1,418 jobs in 1,895.16 seconds of recorded execution time; all raw results and the independent offline verifier are retained.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" s="6" customFormat="1" ht="290.3999938964844" hidden="0" customHeight="1">
@@ -792,6 +792,6 @@
     <x:mergeCell ref="A2:B4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb47e2a24c2ad4be1"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81246a98d07b40ab"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Freeze expanded source audit and add bounded BubR1 TPR reanalysis
</commit_message>
<xml_diff>
--- a/submissions/adriamasnou_methods_description.xlsx
+++ b/submissions/adriamasnou_methods_description.xlsx
@@ -671,7 +671,7 @@
     <x:row r="2" s="6" customFormat="1" ht="70" customHeight="1">
       <x:c r="A2" s="5" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Please submit your answers with your Track 2 report. All questions are voluntary; however, submissions without a methods description may be judged less favorably on the Scientific Rigor and Innovation criteria, since the panel can't assess what it can't see. Track 2 accepts one final submission per team.</x:t>
+          <x:t xml:space="preserve">Please submit your answers with your Track 2 report. All questions are voluntary; however, submissions without a methods description may be judged less favorably on the Scientific Rigor and Innovation criteria, since the panel can't assess what it can't see. Organizer update, 23 October 2026: Track 2 permits up to three submissions, with only the latest evaluated and one submitter per team.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -734,14 +734,14 @@
         <x:v>Public drug/target resources and published literature were used for repurposing evidence; no proprietary drug-target database was used. Some published full texts were accessed through institutional subscriptions. Separately, the challenge's gated patient sequencing and clinical material informed the variant analysis under challenge terms. Those restricted inputs are not redistributed. Public-data derivatives used by the navigator and canary are clearly separated from patient-scale inputs.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" s="6" customFormat="1" ht="211.1999969482422" hidden="0" customHeight="1">
+    <x:row r="12" s="6" customFormat="1" ht="224.4" hidden="0" customHeight="1">
       <x:c r="A12" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Please describe the public data sources used in detail (e.g., DrugBank, ChEMBL, ClinicalTrials.gov, OMIM, PubMed literature search).</x:t>
         </x:is>
       </x:c>
       <x:c r="B12" s="8" t="str">
-        <x:v>Crossref reference deposits and local GROBID parsing for source-pyramid discovery; PubMed, Europe PMC and NCBI E-utilities for literature and identifier checks; FDA DailyMed and EMA assessments for regulatory/pharmacology context; ClinVar, gnomAD v4.1, UniProt O60566, OMIM and LOVD for variant/gene evidence; Ensembl VEP, local SpliceAI and Exomiser/HPO for annotation and prioritisation; NIST GIAB HG002/HG001 v4.2.1 GRCh38, Ensembl 116 exons and Phenopacket Store 0.1.19 for a frozen twelve-case, four-arm semi-synthetic evaluation, plus a separately reconstructed FGFR2 scale example. Both 48-job genome-background batches completed. With original HPO, source-gene top-1/5/10 counts were 6/7/8 of nine primary labels on HG002 and 7/8/8 on HG001. They are the same nine labels, not eighteen independent cases. Five labels retain source qualifications; PAX4 and two X cases remain separate. All four phenotype arms and exact-allele evidence are retained in public-validation.md. The separate original-HPO-only comparator ranked 4/8/8 of nine source genes within 1/5/10 among 19,192 gene-symbol records (19,116 Entrez IDs; collapsing shared IDs leaves target ranks unchanged); its different candidate universe prevents a causal estimate of sequencing value. This is constructed source-label recovery, not clinical accuracy. A separate compact source-label extension completed 1,418 jobs across 713 signatures, with a fixed autosomal primary denominator of 681. Original-HPO top-1 was 556/681 versus 430/681 without HPO after a disclosed serialization-parser correction; both evaluations are retained. Ten constructed hypotheses per case, current database knowledge and 321 unread source papers prevent clinical-accuracy or competitor-superiority claims. See compact-public-validation.md. The PGT-M navigator uses the HFEA workbook dated 2026-08-05 plus retained ClinVar gene_condition_source_id, HPO genes_to_disease and OMIM mim2gene files. Source SHA-256 hashes, dates and mapping disagreements are supplied. The expert-assertion proxy uses a dated ClinVar variant_summary snapshot. None of these is described as a live registry mirror.</x:v>
+        <x:v>Crossref reference deposits and local GROBID parsing for source-pyramid discovery; PubMed, Europe PMC and NCBI E-utilities for literature and identifier checks; FDA DailyMed and EMA assessments for regulatory/pharmacology context; ClinVar, gnomAD v4.1, UniProt O60566, OMIM and LOVD for variant/gene evidence; Ensembl VEP, local SpliceAI and Exomiser/HPO for annotation and prioritisation; NIST GIAB HG002/HG001 v4.2.1 GRCh38, Ensembl 116 exons and Phenopacket Store 0.1.19 for a frozen twelve-case, four-arm semi-synthetic evaluation, plus a separately reconstructed FGFR2 scale example. Both 48-job genome-background batches completed. With original HPO, source-gene top-1/5/10 counts were 6/7/8 of nine primary labels on HG002 and 7/8/8 on HG001. They are the same nine labels, not eighteen independent cases. Five labels retain source qualifications; PAX4 and two X cases remain separate. All four phenotype arms and exact-allele evidence are retained in public-validation.md. The separate original-HPO-only comparator ranked 4/8/8 of nine source genes within 1/5/10 among 19,192 gene-symbol records (19,116 Entrez IDs; collapsing shared IDs leaves target ranks unchanged); its different candidate universe prevents a causal estimate of sequencing value. This is constructed source-label recovery, not clinical accuracy. A separate compact source-label extension completed 1,418 jobs across 713 signatures, with a fixed autosomal primary denominator of 681. Original-HPO top-1 was 556/681 versus 430/681 without HPO after a disclosed serialization-parser correction; both evaluations are retained. Ten constructed hypotheses per case and current database knowledge prevent clinical-accuracy or competitor-superiority claims. Source review remains incomplete: the frozen post-inference snapshot at 18:00 UTC on 24 October 2026 records 178/334 full-main-text reviews, 80 complete paper reviews, 843/1,389 adjudicated packet mappings and 187/713 fully source-audited case signatures. See compact-public-validation.md. The PGT-M navigator uses the HFEA workbook dated 2026-08-05 plus retained ClinVar gene_condition_source_id, HPO genes_to_disease and OMIM mim2gene files. Source SHA-256 hashes, dates and mapping disagreements are supplied. The expert-assertion proxy uses a dated ClinVar variant_summary snapshot. None of these is described as a live registry mirror.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
Freeze 18:27 source audit and disclose Grok search assistance
</commit_message>
<xml_diff>
--- a/submissions/adriamasnou_methods_description.xlsx
+++ b/submissions/adriamasnou_methods_description.xlsx
@@ -741,7 +741,7 @@
         </x:is>
       </x:c>
       <x:c r="B12" s="8" t="str">
-        <x:v>Crossref reference deposits and local GROBID parsing for source-pyramid discovery; PubMed, Europe PMC and NCBI E-utilities for literature and identifier checks; FDA DailyMed and EMA assessments for regulatory/pharmacology context; ClinVar, gnomAD v4.1, UniProt O60566, OMIM and LOVD for variant/gene evidence; Ensembl VEP, local SpliceAI and Exomiser/HPO for annotation and prioritisation; NIST GIAB HG002/HG001 v4.2.1 GRCh38, Ensembl 116 exons and Phenopacket Store 0.1.19 for a frozen twelve-case, four-arm semi-synthetic evaluation, plus a separately reconstructed FGFR2 scale example. Both 48-job genome-background batches completed. With original HPO, source-gene top-1/5/10 counts were 6/7/8 of nine primary labels on HG002 and 7/8/8 on HG001. They are the same nine labels, not eighteen independent cases. Five labels retain source qualifications; PAX4 and two X cases remain separate. All four phenotype arms and exact-allele evidence are retained in public-validation.md. The separate original-HPO-only comparator ranked 4/8/8 of nine source genes within 1/5/10 among 19,192 gene-symbol records (19,116 Entrez IDs; collapsing shared IDs leaves target ranks unchanged); its different candidate universe prevents a causal estimate of sequencing value. This is constructed source-label recovery, not clinical accuracy. A separate compact source-label extension completed 1,418 jobs across 713 signatures, with a fixed autosomal primary denominator of 681. Original-HPO top-1 was 556/681 versus 430/681 without HPO after a disclosed serialization-parser correction; both evaluations are retained. Ten constructed hypotheses per case and current database knowledge prevent clinical-accuracy or competitor-superiority claims. Source review remains incomplete: the frozen post-inference snapshot at 18:00 UTC on 24 October 2026 records 178/334 full-main-text reviews, 80 complete paper reviews, 843/1,389 adjudicated packet mappings and 187/713 fully source-audited case signatures. See compact-public-validation.md. The PGT-M navigator uses the HFEA workbook dated 2026-08-05 plus retained ClinVar gene_condition_source_id, HPO genes_to_disease and OMIM mim2gene files. Source SHA-256 hashes, dates and mapping disagreements are supplied. The expert-assertion proxy uses a dated ClinVar variant_summary snapshot. None of these is described as a live registry mirror.</x:v>
+        <x:v>Crossref reference deposits and local GROBID parsing for source-pyramid discovery; PubMed, Europe PMC and NCBI E-utilities for literature and identifier checks; FDA DailyMed and EMA assessments for regulatory/pharmacology context; ClinVar, gnomAD v4.1, UniProt O60566, OMIM and LOVD for variant/gene evidence; Ensembl VEP, local SpliceAI and Exomiser/HPO for annotation and prioritisation; NIST GIAB HG002/HG001 v4.2.1 GRCh38, Ensembl 116 exons and Phenopacket Store 0.1.19 for a frozen twelve-case, four-arm semi-synthetic evaluation, plus a separately reconstructed FGFR2 scale example. Both 48-job genome-background batches completed. With original HPO, source-gene top-1/5/10 counts were 6/7/8 of nine primary labels on HG002 and 7/8/8 on HG001. They are the same nine labels, not eighteen independent cases. Five labels retain source qualifications; PAX4 and two X cases remain separate. All four phenotype arms and exact-allele evidence are retained in public-validation.md. The separate original-HPO-only comparator ranked 4/8/8 of nine source genes within 1/5/10 among 19,192 gene-symbol records (19,116 Entrez IDs; collapsing shared IDs leaves target ranks unchanged); its different candidate universe prevents a causal estimate of sequencing value. This is constructed source-label recovery, not clinical accuracy. A separate compact source-label extension completed 1,418 jobs across 713 signatures, with a fixed autosomal primary denominator of 681. Original-HPO top-1 was 556/681 versus 430/681 without HPO after a disclosed serialization-parser correction; both evaluations are retained. Ten constructed hypotheses per case and current database knowledge prevent clinical-accuracy or competitor-superiority claims. Source review remains incomplete: the frozen post-inference snapshot at 18:27 UTC on 24 October 2026 records 210/334 full-main-text reviews, 102 complete paper reviews, 920/1,389 adjudicated packet mappings and 218/713 fully source-audited case signatures. See compact-public-validation.md. The PGT-M navigator uses the HFEA workbook dated 2026-08-05 plus retained ClinVar gene_condition_source_id, HPO genes_to_disease and OMIM mim2gene files. Source SHA-256 hashes, dates and mapping disagreements are supplied. The expert-assertion proxy uses a dated ClinVar variant_summary snapshot. None of these is described as a live registry mirror.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -764,14 +764,14 @@
         <x:v>The findings are BUB1B c.2210T&gt;G (p.Leu737*) and c.3006T&gt;G (p.Asn1002Lys). Phase is inferred. NMD of this exact stop allele and N1002K abundance/function are unmeasured. The proposed mechanism concerns BubR1 stability and non-catalytic chromosome-segregation/checkpoint functions (PMID 20516114, 22698286, 33207204). Abundance-limited, function-limited, mixed and indeterminate states are experimental categories, not assigned diagnoses. In-silico predictions and a low local splice score do not substitute for functional evidence. A previous bulk-WGS mosaicism claim was withdrawn after read-mapping correction. No clinical reclassification or treatment follows from this work alone.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" s="6" customFormat="1" ht="145.1999969482422" hidden="0" customHeight="1">
+    <x:row r="15" s="6" customFormat="1" ht="171.6" hidden="0" customHeight="1">
       <x:c r="A15" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Please provide an estimate of time or effort spent on this analysis (if possible).</x:t>
         </x:is>
       </x:c>
       <x:c r="B15" s="8" t="str">
-        <x:v>One participant with LLM assistance; project records span 2026-08-26 to 2026-10-24, not continuous full-time effort. Total person-hours and cost were not reliably logged. Historical recorded runs include VEP annotation of 313,417 distinct variants in 10 min 28 s and an Exomiser HG002 spike-in run in 9 min 20 s on a local Apple M3 Max laptop with external databases; the new two-job FGFR2 reconstruction completed in 200.48 s including startup, with FGFR2 first among 2 and 471 scored genes. The August configuration was not recovered. The 48-job HG002 and HG001 batches took 3,488.41 and 3,607.42 seconds respectively, including each JVM startup and excluding input preparation/downloads. Their conservative ranks are retained with exact runtime configurations. These are machine-specific observations with different settings, not general runtime or accuracy improvements. Prior records identify Anthropic Claude-assisted work; this revision used OpenAI Codex for research, code, drafting and checks. The participant confirms Claude Max 20x and ChatGPT Pro 200 account tiers (23 October 2026). Provider retention settings have not been independently verified. No claim of human clinical expert review is made. No wet-lab experiment, patient treatment or laboratory commitment has occurred. The separate compact extension completed 1,418 jobs in 1,895.16 seconds of recorded execution time; all raw results and the independent offline verifier are retained.</x:v>
+        <x:v>One participant with LLM assistance; project records span 2026-08-26 to 2026-10-24, not continuous full-time effort. Total person-hours and cost were not reliably logged. Historical recorded runs include VEP annotation of 313,417 distinct variants in 10 min 28 s and an Exomiser HG002 spike-in run in 9 min 20 s on a local Apple M3 Max laptop with external databases; the new two-job FGFR2 reconstruction completed in 200.48 s including startup, with FGFR2 first among 2 and 471 scored genes. The August configuration was not recovered. The 48-job HG002 and HG001 batches took 3,488.41 and 3,607.42 seconds respectively, including each JVM startup and excluding input preparation/downloads. Their conservative ranks are retained with exact runtime configurations. These are machine-specific observations with different settings, not general runtime or accuracy improvements. Prior records identify Anthropic Claude-assisted work; this revision used OpenAI Codex for research, code, drafting and checks. The participant confirms Claude Max 20x and ChatGPT Pro 200 account tiers (23 October 2026). Provider retention settings have not been independently verified. No claim of human clinical expert review is made. No wet-lab experiment, patient treatment or laboratory commitment has occurred. The separate compact extension completed 1,418 jobs in 1,895.16 seconds of recorded execution time; all raw results and the independent offline verifier are retained. On 24 October, xAI Grok in Expert mode assisted public literature-access and official-rule searches. Its account tier was not independently verified. Outputs were treated as leads requiring primary-source verification before adoption; no controlled challenge data was sent to Grok.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" s="6" customFormat="1" ht="290.3999938964844" hidden="0" customHeight="1">

</xml_diff>